<commit_message>
add work hours in timesheet
</commit_message>
<xml_diff>
--- a/Week_3/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_3/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
   <si>
     <t>Week_1</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t>Wireframe in Figma (Hospital NavBar, Hero Section, specialties)</t>
+  </si>
+  <si>
+    <t>Wireframe in Figma (Add Doctor section and deatils)</t>
   </si>
 </sst>
 </file>
@@ -2009,9 +2012,15 @@
     </row>
     <row r="42" spans="1:27" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A42" s="25"/>
-      <c r="B42" s="25"/>
-      <c r="C42" s="25"/>
-      <c r="D42" s="25"/>
+      <c r="B42" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="C42" s="27">
+        <v>46054</v>
+      </c>
+      <c r="D42" s="25">
+        <v>2.75</v>
+      </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
@@ -2392,7 +2401,7 @@
       <c r="C55" s="22"/>
       <c r="D55" s="22">
         <f>SUM(D39:D53)</f>
-        <v>5.4</v>
+        <v>8.15</v>
       </c>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>

</xml_diff>

<commit_message>
update hours in timesheet
</commit_message>
<xml_diff>
--- a/Week_3/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
+++ b/Week_3/HTTP 5310 – Capstone Timesheet_Ripal Patel.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="39">
   <si>
     <t>Week_1</t>
   </si>
@@ -130,6 +130,12 @@
   </si>
   <si>
     <t>Wireframe in Figma (Add Doctor section and deatils)</t>
+  </si>
+  <si>
+    <t>Wireframe in Figma (Home page - created)</t>
+  </si>
+  <si>
+    <t>Week_3</t>
   </si>
 </sst>
 </file>
@@ -1870,7 +1876,7 @@
     </row>
     <row r="38" spans="1:27" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A38" s="20" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="B38" s="20" t="s">
         <v>1</v>
@@ -2047,9 +2053,15 @@
     </row>
     <row r="43" spans="1:27" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A43" s="25"/>
-      <c r="B43" s="25"/>
-      <c r="C43" s="25"/>
-      <c r="D43" s="25"/>
+      <c r="B43" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="C43" s="27">
+        <v>46055</v>
+      </c>
+      <c r="D43" s="25">
+        <v>3.75</v>
+      </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
@@ -2401,7 +2413,7 @@
       <c r="C55" s="22"/>
       <c r="D55" s="22">
         <f>SUM(D39:D53)</f>
-        <v>8.15</v>
+        <v>11.9</v>
       </c>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>

</xml_diff>